<commit_message>
committing the batch and shell script which seem to have changed, but in an unclear way; I re-downloaded them from main so we can have these straight for subsequent merge of updated code
</commit_message>
<xml_diff>
--- a/process/configuration/assets/output_data_dictionary.xlsx
+++ b/process/configuration/assets/output_data_dictionary.xlsx
@@ -1408,4 +1408,231 @@
     <oddHeader>&amp;C&amp;"Calibri"&amp;12&amp;KEEDC00 RMIT Classification: Trusted&amp;1#_x000D_</oddHeader>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E46915CC77A6414794C0659BE0416FBE" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ce73daeef664d7c8d016e21b47135507">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d026c80c-8c89-4d76-b5a4-adafffa27ea9" xmlns:ns3="0f2f1471-5c80-47c6-b5fc-5f7f410df7a8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6117017243beacc659db0547db5dd191" ns2:_="" ns3:_="">
+    <xsd:import namespace="d026c80c-8c89-4d76-b5a4-adafffa27ea9"/>
+    <xsd:import namespace="0f2f1471-5c80-47c6-b5fc-5f7f410df7a8"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d026c80c-8c89-4d76-b5a4-adafffa27ea9" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="14" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="16" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="c921d02d-b337-4ce5-bd1c-22d9132a6b17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="18" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="0f2f1471-5c80-47c6-b5fc-5f7f410df7a8" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="17" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3898acd8-9e76-4e3a-bd5c-f786070581b8}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="0f2f1471-5c80-47c6-b5fc-5f7f410df7a8">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d026c80c-8c89-4d76-b5a4-adafffa27ea9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="0f2f1471-5c80-47c6-b5fc-5f7f410df7a8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90EF6D81-00BC-4493-8292-A3D18C3BBB5F}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC38DB0F-9330-4BF2-B8E8-1ED662DF4A97}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BB74974-DA4A-4929-985E-3BC9CEF37435}"/>
 </file>
</xml_diff>

<commit_message>
draft approach for Mexicali DENUE based analyses
</commit_message>
<xml_diff>
--- a/process/configuration/assets/output_data_dictionary.xlsx
+++ b/process/configuration/assets/output_data_dictionary.xlsx
@@ -425,13 +425,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D96"/>
+  <dimension ref="A1:F105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="92" customWidth="1" min="2" max="2"/>
     <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -452,6 +454,16 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Statistic</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Scale</t>
         </is>
       </c>
@@ -472,7 +484,13 @@
           <t>Continent</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>city</t>
         </is>
@@ -494,7 +512,13 @@
           <t>Country</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>city</t>
         </is>
@@ -516,7 +540,13 @@
           <t>ISO 3166-1 alpha-2</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>city</t>
         </is>
@@ -538,7 +568,13 @@
           <t>study_region</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>city, grid</t>
         </is>
@@ -562,6 +598,16 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>km²</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>sum</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>city</t>
         </is>
       </c>
@@ -584,6 +630,16 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>persons</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>sum</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>city</t>
         </is>
       </c>
@@ -606,6 +662,16 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>persons per km²</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>rate</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>city</t>
         </is>
       </c>
@@ -628,6 +694,16 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>city</t>
         </is>
       </c>
@@ -650,6 +726,16 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>count per km²</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>rate</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>city</t>
         </is>
       </c>
@@ -672,6 +758,16 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>km²</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>sum</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>grid, custom areas</t>
         </is>
       </c>
@@ -694,6 +790,16 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
+          <t>persons</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>sum</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>grid, custom areas</t>
         </is>
       </c>
@@ -716,6 +822,16 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>persons per km²</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>rate</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>grid, custom areas</t>
         </is>
       </c>
@@ -738,6 +854,16 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>grid, custom areas</t>
         </is>
       </c>
@@ -760,6 +886,16 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
+          <t>count per km²</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>rate</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>grid, custom areas</t>
         </is>
       </c>
@@ -782,6 +918,16 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>city, grid</t>
         </is>
       </c>
@@ -802,7 +948,13 @@
           <t>grid_id</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
         <is>
           <t>grid, sample point</t>
         </is>
@@ -824,7 +976,13 @@
           <t>point_id</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
         <is>
           <t>sample point</t>
         </is>
@@ -848,6 +1006,16 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>custom areas</t>
         </is>
       </c>
@@ -860,7 +1028,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>The destination whose access is measured.  The default destinations are listed below.  Walking and cycling access draw on the same destination definitions; cycling additionally pairs a strict and a lenient variant of each core category (food, public open space, public transport) so that composite "all categories reachable" indicators can be derived per variant.</t>
+          <t>The destination whose access is measured.  The default destinations are listed below.  Walking and cycling access draw on the same destination definitions, declared once in a region's "accessibility" configuration; each pairs a strict and a lenient variant of each core category (food, public open space, public transport) so that composite "all categories reachable" indicators can be derived per variant.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -869,6 +1037,8 @@
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -886,7 +1056,9 @@
           <t>fresh_food_market</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
         <is>
           <t>Food (strict)</t>
         </is>
@@ -908,7 +1080,9 @@
           <t>fresh_food_pooled</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
         <is>
           <t>Food (lenient)</t>
         </is>
@@ -930,7 +1104,9 @@
           <t>convenience</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
         <is>
           <t>Food</t>
         </is>
@@ -952,7 +1128,9 @@
           <t>public_open_space_large</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
         <is>
           <t>Open space (strict)</t>
         </is>
@@ -974,7 +1152,9 @@
           <t>public_open_space_any</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
         <is>
           <t>Open space (lenient)</t>
         </is>
@@ -996,7 +1176,9 @@
           <t>large_public_green_space</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
         <is>
           <t>Open space</t>
         </is>
@@ -1018,7 +1200,9 @@
           <t>pt_frequent</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
         <is>
           <t>Transport (strict, cycling)</t>
         </is>
@@ -1040,7 +1224,9 @@
           <t>pt_gtfs_freq_20</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
         <is>
           <t>Transport (walking)</t>
         </is>
@@ -1062,7 +1248,9 @@
           <t>pt_gtfs_freq_30</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
         <is>
           <t>Transport (walking)</t>
         </is>
@@ -1084,7 +1272,9 @@
           <t>pt_gtfs_any</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
         <is>
           <t>Transport</t>
         </is>
@@ -1106,7 +1296,9 @@
           <t>pt_osm_any</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
         <is>
           <t>Transport</t>
         </is>
@@ -1128,7 +1320,9 @@
           <t>pt_any</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
         <is>
           <t>Transport (lenient)</t>
         </is>
@@ -1150,7 +1344,9 @@
           <t>all_strict</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
         <is>
           <t>Combined</t>
         </is>
@@ -1172,7 +1368,9 @@
           <t>all_lenient</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
         <is>
           <t>Combined</t>
         </is>
@@ -1194,7 +1392,9 @@
           <t>activity_centre_local</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
         <is>
           <t>Derived</t>
         </is>
@@ -1216,7 +1416,9 @@
           <t>activity_centre_complete</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
         <is>
           <t>Derived</t>
         </is>
@@ -1235,6 +1437,8 @@
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1244,7 +1448,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Distance threshold (m).  Distances can be customised to locally policy-relevant values.  Walking access uses the configured neighbourhood accessibility threshold (default 500 m); cycling access is evaluated at each configured cycling distance (defaults: 500 m, 1000 m, 2000 m and 5000 m), so a cycling access variable exists for each distance.</t>
+          <t>Distance threshold (m).  Distances can be customised to locally policy-relevant values.  The core walking access indicators use the configured neighbourhood accessibility threshold (default 500 m).  Where a region configures the optional pedestrian accessibility analysis, walking access is additionally evaluated at each configured pedestrian distance, and cycling access at each configured cycling distance (defaults: 500 m, 1000 m, 2000 m and 5000 m), so an access variable exists for each distance.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1253,6 +1457,8 @@
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1271,6 +1477,8 @@
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1290,6 +1498,16 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
+          <t>score 0-1</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
           <t>sample point</t>
         </is>
       </c>
@@ -1312,6 +1530,16 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
+          <t>metres</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
           <t>sample point</t>
         </is>
       </c>
@@ -1334,6 +1562,16 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
           <t>grid, custom areas</t>
         </is>
       </c>
@@ -1356,6 +1594,16 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
           <t>city, custom areas</t>
         </is>
       </c>
@@ -1363,20 +1611,30 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (walking)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Average population density of the local walkable neighbourhood (population per km², based on the population grid cells intersecting the sample point neighbourhood)</t>
+          <t>Score (0/1): the destination is reachable within [x] m along the pedestrian network</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>sp_local_nh_avg_pop_density</t>
+          <t>sp_walk_access_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
+        <is>
+          <t>score 0-1</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
         <is>
           <t>sample point</t>
         </is>
@@ -1385,20 +1643,30 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (walking)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Average street intersection density of the local walkable neighbourhood (intersections per km²)</t>
+          <t>Distance (m) along the pedestrian network to the nearest destination</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>sp_local_nh_avg_intersection_density</t>
+          <t>sp_walk_nearest_node_[destination]</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
+        <is>
+          <t>metres</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
         <is>
           <t>sample point</t>
         </is>
@@ -1407,152 +1675,222 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (walking)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Daily living score (/3): sum of access scores for fresh food, convenience and public transport destinations</t>
+          <t>Percentage of population with walking access within [x] m to the destination</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>sp_daily_living_score</t>
+          <t>pct_access_walk_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>sample point</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (walking)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Walkability index: sum of z-scores of the daily living score, neighbourhood population density and neighbourhood intersection density</t>
+          <t>Percentage of population with walking access within [x] m to the destination (population weighted)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>sp_walkability_index</t>
+          <t>pop_pct_access_walk_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>sample point</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (walking)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Average walkable neighbourhood population density (population per km²) of sample points in this area</t>
+          <t>Average distance (m) along the pedestrian network to the nearest destination</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>local_nh_population_density</t>
+          <t>avg_walk_dist_[destination]</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>grid, city, custom areas</t>
+          <t>metres</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (walking)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Average walkable neighbourhood intersection density (intersections per km²) of sample points in this area</t>
+          <t>Average distance (m) along the pedestrian network to the nearest destination (population weighted)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>local_nh_intersection_density</t>
+          <t>pop_avg_walk_dist_[destination]</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>grid, city, custom areas</t>
+          <t>metres</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (walking)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Average daily living score (/3) of sample points in this area</t>
+          <t>Score (0/1): the nearest destination is further than [x] m along the pedestrian network</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>local_daily_living</t>
+          <t>sp_walk_beyond_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>grid, city, custom areas</t>
+          <t>score 0-1</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>sample point</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (walking)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Average walkability index of sample points in this area</t>
+          <t>Percentage of population living further than [x] m along the pedestrian network from the nearest destination</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>local_walkability</t>
+          <t>pct_beyond_walk_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>grid, city, custom areas</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (walking)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Average walkable neighbourhood population density (population per km²; population weighted)</t>
+          <t>Percentage of population living further than [x] m along the pedestrian network from the nearest destination (population weighted)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>pop_nh_pop_density</t>
+          <t>pop_pct_beyond_walk_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
         <is>
           <t>city, custom areas</t>
         </is>
@@ -1566,17 +1904,27 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Average walkable neighbourhood intersection density (intersections per km²; population weighted)</t>
+          <t>Average population density of the local walkable neighbourhood (population per km², based on the population grid cells intersecting the sample point neighbourhood)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>pop_nh_intersection_density</t>
+          <t>sp_local_nh_avg_pop_density</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>city, custom areas</t>
+          <t>persons per km²</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>sample point</t>
         </is>
       </c>
     </row>
@@ -1588,17 +1936,27 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Average daily living score (/3; population weighted)</t>
+          <t>Average street intersection density of the local walkable neighbourhood (intersections per km²)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>pop_daily_living</t>
+          <t>sp_local_nh_avg_intersection_density</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>city, custom areas</t>
+          <t>count per km²</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>sample point</t>
         </is>
       </c>
     </row>
@@ -1610,37 +1968,57 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Average walkability index (population weighted)</t>
+          <t>Daily living score (/3): sum of access scores for fresh food, convenience and public transport destinations</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>pop_walkability</t>
+          <t>sp_daily_living_score</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>city, custom areas</t>
+          <t>score 0-3</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>sample point</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Indicator estimates: cycling accessibility</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Score (0/1): the destination is reachable within [x] m by cycling, routed using the [network] measure</t>
+          <t>Walkability index: sum of z-scores of the daily living score, neighbourhood population density and neighbourhood intersection density</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>sp_cycle_[network]access_[destination]_[x]m</t>
+          <t>sp_walkability_index</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
+        <is>
+          <t>index (sum of z-scores)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
         <is>
           <t>sample point</t>
         </is>
@@ -1649,108 +2027,158 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Indicator estimates: cycling accessibility</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Distance (m) by cycling to the nearest destination, routed using the [network] measure</t>
+          <t>Average walkable neighbourhood population density (population per km²) of sample points in this area</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>sp_cycle_[network]nearest_node_[destination]</t>
+          <t>local_nh_population_density</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>sample point</t>
+          <t>persons per km²</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Indicator estimates: cycling accessibility</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Percentage of population with cycling access within [x] m to the destination, routed using the [network] measure</t>
+          <t>Average walkable neighbourhood intersection density (intersections per km²) of sample points in this area</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>pct_access_cycle_[network][destination]_[x]m</t>
+          <t>local_nh_intersection_density</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>grid, custom areas</t>
+          <t>count per km²</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Indicator estimates: cycling accessibility</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Percentage of population with cycling access within [x] m to the destination, routed using the [network] measure (population weighted)</t>
+          <t>Average daily living score (/3) of sample points in this area</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>pop_pct_access_cycle_[network][destination]_[x]m</t>
+          <t>local_daily_living</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>city, custom areas</t>
+          <t>score 0-3</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Indicator estimates: cycling accessibility</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Average distance (m) by cycling to the nearest destination, routed using the [network] measure</t>
+          <t>Average walkability index of sample points in this area</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>avg_cycle_dist_[network][destination]</t>
+          <t>local_walkability</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>grid, custom areas</t>
+          <t>index (sum of z-scores)</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Indicator estimates: cycling accessibility</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Average distance (m) by cycling to the nearest destination, routed using the [network] measure (population weighted)</t>
+          <t>Average walkable neighbourhood population density (population per km²; population weighted)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>pop_avg_cycle_dist_[network][destination]</t>
+          <t>pop_nh_pop_density</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
+        <is>
+          <t>persons per km²</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
         <is>
           <t>city, custom areas</t>
         </is>
@@ -1759,198 +2187,288 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Heat Exposure Index (HEI): the heat exposure sub-index, derived from land surface temperature</t>
+          <t>Average walkable neighbourhood intersection density (intersections per km²; population weighted)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>urban_heat_exposure_index</t>
+          <t>pop_nh_intersection_density</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>count per km²</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Land surface temperature (°C): the temperature of the Earth’s surface, indicating the lived experience of heat (Landsat 8 surface reflectance, hottest third of the year)</t>
+          <t>Average daily living score (/3; population weighted)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>urban_heat_land_surface_temp_c</t>
+          <t>pop_daily_living</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>score 0-3</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Heat Sensitivity Index (HSI): the equally weighted heat sensitivity sub-index of land surface albedo, NDVI, NDBI, local climate zone, population density and vulnerable population</t>
+          <t>Average walkability index (population weighted)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>urban_heat_sensitivity_index</t>
+          <t>pop_walkability</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>index (sum of z-scores)</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: cycling accessibility</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Land surface albedo: solar reflectance, where higher reflectance implies less surface heat retention (inverted, so that higher values indicate greater heat vulnerability)</t>
+          <t>Score (0/1): the destination is reachable within [x] m by cycling, routed using the [network] measure</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>urban_heat_land_surface_albedo</t>
+          <t>sp_cycle_[network]access_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>score 0-1</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>sample point</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: cycling accessibility</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Normalised Difference Vegetation Index (NDVI): a spectral index of vegetation health and greenness (inverted, so that higher values indicate greater heat vulnerability)</t>
+          <t>Distance (m) by cycling to the nearest destination, routed using the [network] measure</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>urban_heat_ndvi</t>
+          <t>sp_cycle_[network]nearest_node_[destination]</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>metres</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>sample point</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: cycling accessibility</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Normalised Difference Built-up Index (NDBI): a spectral index of impervious surfaces such as concrete and asphalt</t>
+          <t>Percentage of population with cycling access within [x] m to the destination, routed using the [network] measure</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>urban_heat_ndbi</t>
+          <t>pct_access_cycle_[network][destination]_[x]m</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: cycling accessibility</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Local Climate Zone: a standardised classification of land cover typologies for urban heat island studies, ordered from least heat retaining (water) to most heat retaining (bare rock or paved)</t>
+          <t>Percentage of population with cycling access within [x] m to the destination, routed using the [network] measure (population weighted)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>urban_heat_local_climate_zone_ordered</t>
+          <t>pop_pct_access_cycle_[network][destination]_[x]m</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: cycling accessibility</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Population density (persons per km²), from the GHS-POP global human settlement population grid</t>
+          <t>Average distance (m) by cycling to the nearest destination, routed using the [network] measure</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>urban_heat_population_density_per_sqkm</t>
+          <t>avg_cycle_dist_[network][destination]</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>metres</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: cycling accessibility</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Vulnerable population (%): those most at risk from heat on the basis of age, being the combined proportion of the population aged 0–4 and 65+ years</t>
+          <t>Average distance (m) by cycling to the nearest destination, routed using the [network] measure (population weighted)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>urban_heat_vulnerable_pop_pct</t>
+          <t>pop_avg_cycle_dist_[network][destination]</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>metres</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
@@ -1962,15 +2480,25 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Adaptive Capability Index (ACI): the equally weighted adaptive capability sub-index of child dependency ratio, subnational Human Development Index and infant mortality rate; higher values indicate lower adaptive capability</t>
+          <t>Heat Exposure Index (HEI): the heat exposure sub-index, derived from land surface temperature</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>urban_heat_adaptive_capability_index</t>
+          <t>urban_heat_exposure_index</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
+        <is>
+          <t>index 0-1</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
         <is>
           <t>sample point, grid, city, custom areas</t>
         </is>
@@ -1984,15 +2512,25 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Child dependency ratio: children (aged 0–14 years) relative to the working age population (15–64 years), indicating economic reliance</t>
+          <t>Land surface temperature (°C): the temperature of the Earth’s surface, indicating the lived experience of heat (Landsat 8 surface reflectance, hottest third of the year)</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>urban_heat_child_dependency_ratio</t>
+          <t>urban_heat_land_surface_temp_c</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
+        <is>
+          <t>degrees Celsius</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
         <is>
           <t>sample point, grid, city, custom areas</t>
         </is>
@@ -2006,15 +2544,25 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Subnational Human Development Index: human well-being assessed through education, health and standard of living</t>
+          <t>Heat Sensitivity Index (HSI): the equally weighted heat sensitivity sub-index of land surface albedo, NDVI, NDBI, local climate zone, population density and vulnerable population</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>urban_heat_subnational_hdi</t>
+          <t>urban_heat_sensitivity_index</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
+        <is>
+          <t>index 0-1</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
         <is>
           <t>sample point, grid, city, custom areas</t>
         </is>
@@ -2028,15 +2576,25 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Infant mortality rate: deaths of children under 1 year of age per 1000 live births, a key indicator of population health</t>
+          <t>Land surface albedo: solar reflectance, where higher reflectance implies less surface heat retention (inverted, so that higher values indicate greater heat vulnerability)</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>urban_heat_infant_mortality_rate</t>
+          <t>urban_heat_land_surface_albedo</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
+        <is>
+          <t>proportion 0-1</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
         <is>
           <t>sample point, grid, city, custom areas</t>
         </is>
@@ -2050,15 +2608,25 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Global Urban Heat Vulnerability Index (GUHVI): the equally weighted composite of the Heat Exposure, Heat Sensitivity and Adaptive Capability indices, (HEI + HSI + ACI) / 3</t>
+          <t>Normalised Difference Vegetation Index (NDVI): a spectral index of vegetation health and greenness (inverted, so that higher values indicate greater heat vulnerability)</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>urban_heat_guhvi</t>
+          <t>urban_heat_ndvi</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
+        <is>
+          <t>index -1 to 1</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
         <is>
           <t>sample point, grid, city, custom areas</t>
         </is>
@@ -2072,15 +2640,25 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Global Urban Heat Vulnerability Index (GUHVI) class, from 1 (least vulnerable) to 5 (most vulnerable)</t>
+          <t>Normalised Difference Built-up Index (NDBI): a spectral index of impervious surfaces such as concrete and asphalt</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>urban_heat_guhvi_class</t>
+          <t>urban_heat_ndbi</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
+        <is>
+          <t>index -1 to 1</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
         <is>
           <t>sample point, grid, city, custom areas</t>
         </is>
@@ -2094,215 +2672,315 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Percentage of population in Global Urban Heat Vulnerability Index (GUHVI) class 5, the most vulnerable class</t>
+          <t>Local Climate Zone: a standardised classification of land cover typologies for urban heat island studies, ordered from least heat retaining (water) to most heat retaining (bare rock or paved)</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>pct_urban_heat_guhvi_class_5_most_vulnerable</t>
+          <t>urban_heat_local_climate_zone_ordered</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>grid, city, custom areas</t>
+          <t>ordered class</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Timepoint label of the observation (e.g. year)</t>
+          <t>Population density (persons per km²), from the GHS-POP global human settlement population grid</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>timepoint</t>
+          <t>urban_heat_population_density_per_sqkm</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>persons per km²</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Output variable name of the indicator observed (see the indicator entries of this data dictionary)</t>
+          <t>Vulnerable population (%): those most at risk from heat on the basis of age, being the combined proportion of the population aged 0–4 and 65+ years</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>indicator</t>
+          <t>urban_heat_vulnerable_pop_pct</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Value of the indicator at this timepoint for this unit</t>
+          <t>Adaptive Capability Index (ACI): the equally weighted adaptive capability sub-index of child dependency ratio, subnational Human Development Index and infant mortality rate; higher values indicate lower adaptive capability</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>urban_heat_adaptive_capability_index</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>index 0-1</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Custom area identifier (area panels)</t>
+          <t>Child dependency ratio: children (aged 0–14 years) relative to the working age population (15–64 years), indicating economic reliance</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>area_id</t>
+          <t>urban_heat_child_dependency_ratio</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Unit identifier (generic panels)</t>
+          <t>Subnational Human Development Index: human well-being assessed through education, health and standard of living</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>unit_id</t>
+          <t>urban_heat_subnational_hdi</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>index 0-1</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Baseline timepoint label of the comparison pair</t>
+          <t>Infant mortality rate: deaths of children under 1 year of age per 1000 live births, a key indicator of population health</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>t0</t>
+          <t>urban_heat_infant_mortality_rate</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>deaths per 1,000 live births</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Follow-up timepoint label of the comparison pair</t>
+          <t>Global Urban Heat Vulnerability Index (GUHVI): the equally weighted composite of the Heat Exposure, Heat Sensitivity and Adaptive Capability indices, (HEI + HSI + ACI) / 3</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>t1</t>
+          <t>urban_heat_guhvi</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>index 0-1</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Indicator value at the baseline timepoint</t>
+          <t>Global Urban Heat Vulnerability Index (GUHVI) class, from 1 (least vulnerable) to 5 (most vulnerable)</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>value_t0</t>
+          <t>urban_heat_guhvi_class</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>class 1-5</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Indicator value at the follow-up timepoint</t>
+          <t>Percentage of population in Global Urban Heat Vulnerability Index (GUHVI) class 5, the most vulnerable class</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>value_t1</t>
+          <t>pct_urban_heat_guhvi_class_5_most_vulnerable</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>grid, city, custom areas</t>
         </is>
       </c>
     </row>
@@ -2314,15 +2992,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Change metric: 'pp_change' (percentage point change; used for bounded percentage indicators), 'diff' (absolute difference) or 'pct_change' (relative change, %, masked where the baseline is zero)</t>
+          <t>Timepoint label of the observation (e.g. year)</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>metric</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
+          <t>timepoint</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
         <is>
           <t>longitudinal series</t>
         </is>
@@ -2336,15 +3016,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Change in the indicator between t0 and t1, as per the change metric</t>
+          <t>Output variable name of the indicator observed (see the indicator entries of this data dictionary)</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>change</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
+          <t>indicator</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr">
         <is>
           <t>longitudinal series</t>
         </is>
@@ -2358,15 +3040,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Whether a policy review checklist was configured and scored for this timepoint</t>
+          <t>Value of the indicator at this timepoint for this unit</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>assessed</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
+          <t>value</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr">
         <is>
           <t>longitudinal series</t>
         </is>
@@ -2380,15 +3064,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Policy review checklist version</t>
+          <t>Custom area identifier (area panels)</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>checklist_version</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
+          <t>area_id</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
         <is>
           <t>longitudinal series</t>
         </is>
@@ -2402,15 +3088,17 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Count of policies identified as present in the policy review</t>
+          <t>Unit identifier (generic panels)</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>presence_numerator</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
+          <t>unit_id</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
         <is>
           <t>longitudinal series</t>
         </is>
@@ -2424,15 +3112,17 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Number of policies assessed for presence in the policy review</t>
+          <t>Baseline timepoint label of the comparison pair</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>presence_denominator</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
+          <t>t0</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
         <is>
           <t>longitudinal series</t>
         </is>
@@ -2446,15 +3136,17 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Policy presence score (%)</t>
+          <t>Follow-up timepoint label of the comparison pair</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>presence_pct</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
+          <t>t1</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
         <is>
           <t>longitudinal series</t>
         </is>
@@ -2468,15 +3160,17 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Sum of policy quality scores in the policy review</t>
+          <t>Indicator value at the baseline timepoint</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>quality_numerator</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
+          <t>value_t0</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
         <is>
           <t>longitudinal series</t>
         </is>
@@ -2490,15 +3184,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Maximum possible sum of policy quality scores in the policy review</t>
+          <t>Indicator value at the follow-up timepoint</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>quality_denominator</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
+          <t>value_t1</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
         <is>
           <t>longitudinal series</t>
         </is>
@@ -2512,15 +3208,233 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
+          <t>Change metric: 'pp_change' (percentage point change; used for bounded percentage indicators), 'diff' (absolute difference) or 'pct_change' (relative change, %, masked where the baseline is zero)</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Change in the indicator between t0 and t1, as per the change metric</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>change</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Whether a policy review checklist was configured and scored for this timepoint</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>assessed</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Policy review checklist version</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>checklist_version</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Count of policies identified as present in the policy review</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>presence_numerator</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Number of policies assessed for presence in the policy review</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>presence_denominator</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Policy presence score (%)</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>presence_pct</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Sum of policy quality scores in the policy review</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>quality_numerator</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Maximum possible sum of policy quality scores in the policy review</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>quality_denominator</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
           <t>Policy quality score (%)</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C105" t="inlineStr">
         <is>
           <t>quality_pct</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr">
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
         <is>
           <t>longitudinal series</t>
         </is>

</xml_diff>